<commit_message>
Spectrogram feature first implementation
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexis/Codes/clinical-scope/example/demo_database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3608D68-4A65-564A-A5DD-EC72C2C7A843}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB8B003-0A20-C849-ADE4-29F7679108E7}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="26280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19080" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="signals" sheetId="1" r:id="rId1"/>
     <sheet name="loops" sheetId="2" r:id="rId2"/>
+    <sheet name="spectrograms" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="121">
   <si>
     <t>datasource</t>
   </si>
@@ -257,57 +258,57 @@
     <t>Esophageal Press. (cmH2O)</t>
   </si>
   <si>
+    <t>mindray_scope</t>
+  </si>
+  <si>
+    <t>ECG_II</t>
+  </si>
+  <si>
+    <t>ECG II</t>
+  </si>
+  <si>
+    <t>mV</t>
+  </si>
+  <si>
+    <t>#2c3e50</t>
+  </si>
+  <si>
+    <t>Waveform</t>
+  </si>
+  <si>
+    <t>Pleth</t>
+  </si>
+  <si>
+    <t>Plethysmography</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>#7d3c98</t>
+  </si>
+  <si>
+    <t>Art</t>
+  </si>
+  <si>
+    <t>Paw</t>
+  </si>
+  <si>
+    <t>#e67e22</t>
+  </si>
+  <si>
+    <t>Vol</t>
+  </si>
+  <si>
+    <t>#2471a3</t>
+  </si>
+  <si>
+    <t>debit</t>
+  </si>
+  <si>
     <t>Flow</t>
   </si>
   <si>
-    <t>mindray_scope</t>
-  </si>
-  <si>
-    <t>ECG_II</t>
-  </si>
-  <si>
-    <t>ECG II</t>
-  </si>
-  <si>
-    <t>mV</t>
-  </si>
-  <si>
-    <t>#2c3e50</t>
-  </si>
-  <si>
-    <t>Waveform</t>
-  </si>
-  <si>
-    <t>Pleth</t>
-  </si>
-  <si>
-    <t>Plethysmography</t>
-  </si>
-  <si>
-    <t>AU</t>
-  </si>
-  <si>
-    <t>#7d3c98</t>
-  </si>
-  <si>
-    <t>Art</t>
-  </si>
-  <si>
-    <t>Paw</t>
-  </si>
-  <si>
-    <t>#e67e22</t>
-  </si>
-  <si>
-    <t>Vol</t>
-  </si>
-  <si>
-    <t>#2471a3</t>
-  </si>
-  <si>
-    <t>debit</t>
-  </si>
-  <si>
     <t>#1e8449</t>
   </si>
   <si>
@@ -317,6 +318,36 @@
     <t>Port 4 Pressure</t>
   </si>
   <si>
+    <t>other::eeg</t>
+  </si>
+  <si>
+    <t>chan 1</t>
+  </si>
+  <si>
+    <t>EEG 1</t>
+  </si>
+  <si>
+    <t>steelblue</t>
+  </si>
+  <si>
+    <t>chan 2</t>
+  </si>
+  <si>
+    <t>EEG 2</t>
+  </si>
+  <si>
+    <t>darkorange</t>
+  </si>
+  <si>
+    <t>chan 3</t>
+  </si>
+  <si>
+    <t>EEG 3</t>
+  </si>
+  <si>
+    <t>seagreen</t>
+  </si>
+  <si>
     <t>loop_name</t>
   </si>
   <si>
@@ -330,6 +361,30 @@
   </si>
   <si>
     <t>PV loop mindray</t>
+  </si>
+  <si>
+    <t>spectrogram_name</t>
+  </si>
+  <si>
+    <t>freq_min</t>
+  </si>
+  <si>
+    <t>freq_max</t>
+  </si>
+  <si>
+    <t>db_min</t>
+  </si>
+  <si>
+    <t>db_max</t>
+  </si>
+  <si>
+    <t>EEG 1 spectrogram</t>
+  </si>
+  <si>
+    <t>EEG 2 spectrogram</t>
+  </si>
+  <si>
+    <t>EEG 3 spectrogram</t>
   </si>
 </sst>
 </file>
@@ -684,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1244,7 +1299,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
         <v>17</v>
@@ -1258,50 +1313,50 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
         <v>79</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>80</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>81</v>
       </c>
-      <c r="D40" t="s">
+      <c r="I40" t="s">
         <v>82</v>
       </c>
-      <c r="I40" t="s">
+      <c r="N40" t="s">
         <v>83</v>
-      </c>
-      <c r="N40" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" t="s">
         <v>85</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>86</v>
       </c>
-      <c r="D41" t="s">
+      <c r="I41" t="s">
         <v>87</v>
       </c>
-      <c r="I41" t="s">
-        <v>88</v>
-      </c>
       <c r="N41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
         <v>21</v>
@@ -1315,10 +1370,10 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C43" t="s">
         <v>27</v>
@@ -1327,7 +1382,7 @@
         <v>24</v>
       </c>
       <c r="I43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N43" t="s">
         <v>28</v>
@@ -1335,10 +1390,10 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
         <v>30</v>
@@ -1347,7 +1402,7 @@
         <v>31</v>
       </c>
       <c r="I44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N44" t="s">
         <v>30</v>
@@ -1355,13 +1410,13 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B45" t="s">
+        <v>93</v>
+      </c>
+      <c r="C45" t="s">
         <v>94</v>
-      </c>
-      <c r="C45" t="s">
-        <v>78</v>
       </c>
       <c r="D45" t="s">
         <v>75</v>
@@ -1375,7 +1430,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B46" t="s">
         <v>96</v>
@@ -1388,6 +1443,48 @@
       </c>
       <c r="N46" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" t="s">
+        <v>100</v>
+      </c>
+      <c r="I47" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" t="s">
+        <v>102</v>
+      </c>
+      <c r="C48" t="s">
+        <v>103</v>
+      </c>
+      <c r="I48" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>98</v>
+      </c>
+      <c r="B49" t="s">
+        <v>105</v>
+      </c>
+      <c r="C49" t="s">
+        <v>106</v>
+      </c>
+      <c r="I49" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1411,13 +1508,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -1425,7 +1522,7 @@
         <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
         <v>69</v>
@@ -1436,16 +1533,110 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.1640625" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2">
+        <v>0.5</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" t="s">
         <v>102</v>
       </c>
-      <c r="C3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D3" t="s">
-        <v>92</v>
+      <c r="D3">
+        <v>0.5</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4">
+        <v>0.5</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+      <c r="F4">
+        <v>-60</v>
+      </c>
+      <c r="G4">
+        <v>-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixing bad eeg data i nthe example, keep good signals
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -1279,16 +1279,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -1765,6 +1755,12 @@
       <c r="E2" t="n">
         <v>30</v>
       </c>
+      <c r="F2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G2" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1788,6 +1784,12 @@
       <c r="E3" t="n">
         <v>30</v>
       </c>
+      <c r="F3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1812,10 +1814,10 @@
         <v>30</v>
       </c>
       <c r="F4" t="n">
-        <v>-20</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
psd plot type added (issue 73)
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19080" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19080" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="signals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="loops" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="spectrograms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="psds" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1689,7 +1690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18.1640625" customWidth="1" min="2" max="2"/>
@@ -1732,6 +1733,16 @@
           <t>db_max</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>window_s</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>overlap</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1818,6 +1829,233 @@
       </c>
       <c r="G4" t="n">
         <v>85</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.1640625" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>datasource</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>groups</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>signal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>freq_min</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>freq_max</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>db_min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>db_max</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>window_s</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>overlap</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>line_dash</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>edf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EEG PSD (chan 1+2)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>chan 1</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>edf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EEG PSD (chan 1+2)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chan 2</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>edf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EEG PSD (chan 3)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>chan 3</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>edf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EEG PSD (chan 3, window comparison)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>chan 3</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>chan 3 (2s window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>edf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EEG PSD (chan 3, window comparison)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>chan 3</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>chan 3 (8s window)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>darkred</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>dash</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove philips_waves, philips_numerics and syringe datasources (issue 74)
They performed no format-specific parsing, so they were 'other' with extra machinery.
Now that each file in other/ carries its own configuration and time_shift, they no
longer earn a module. Example data moved into other/, configs rekeyed to other::<stem>,
and a folder still named after a removed source is reported with a warning.

Also corrects signal names in the demo workbook that never matched the demo data
(a pre-existing mismatch this migration made visible).
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::waves</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -549,12 +549,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::waves</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ART</t>
+          <t>art</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -576,118 +576,78 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::waves</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PAP</t>
+          <t>pleth</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Esophageal Pressure</t>
+          <t>Plethysmography</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>cmH2O</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>1.35951</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>dash</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Esophageal Pressure</t>
+          <t>AU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::numerics</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P-aer</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Airway Pressure</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>cmH2O</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Pressure &amp; Flow</t>
+          <t>*</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::numerics</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CrbVol</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Heart Rate</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>mL</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>2</v>
+          <t>bpm</t>
+        </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Arterial Pressure</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>philips_waves</t>
+          <t>other::numerics</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CO₂</t>
+          <t>PNId</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CO2</t>
+          <t>Pressure diastolic</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -695,44 +655,68 @@
           <t>mmHg</t>
         </is>
       </c>
+      <c r="H7" t="n">
+        <v>1.5</v>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>CO2</t>
+          <t>Arterial Pressure</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>philips_numerics</t>
+          <t>other::numerics</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>PNIm</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pressure mean</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mmHg</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Arterial Pressure</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>philips_numerics</t>
+          <t>other::numerics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FC</t>
+          <t>PNIs</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Heart Rate</t>
+          <t>Pressure systolic</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>bpm</t>
-        </is>
+          <t>mmHg</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1.5</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -743,111 +727,88 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>philips_numerics</t>
+          <t>other::syringe</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PNId</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Pressure diastolic</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>mmHg</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Arterial Pressure</t>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Europe/Paris</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>philips_numerics</t>
+          <t>other::syringe</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PNIm</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Pressure mean</t>
+          <t>Vitesse Babynoradrenaline</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>mmHg</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Arterial Pressure</t>
-        </is>
+          <t>µg/h</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>philips_numerics</t>
+          <t>eit</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PNIs</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Pressure systolic</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>mmHg</t>
+          <t>*</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Arterial Pressure</t>
+        <v>2.5</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Europe/Paris</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>syringe</t>
+          <t>eit</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Vitesse Babynoradrenaline</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>µg/h</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
+          <t>Ohms</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>EIT Impedance</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -858,18 +819,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Europe/Paris</t>
+          <t>Local 1*</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ohms</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>EIT Impedance</t>
         </is>
       </c>
     </row>
@@ -881,7 +846,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Local 2*</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -891,7 +856,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>black</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -908,7 +873,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Local 1*</t>
+          <t>Local 3*</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -918,7 +883,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -935,7 +900,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Local 2*</t>
+          <t>Local 4*</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -945,7 +910,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>purple</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -962,22 +927,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Local 3*</t>
+          <t>%Local 1*</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ohms</t>
+          <t>Proportion</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>EIT Impedance</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>fraction</t>
         </is>
       </c>
     </row>
@@ -989,22 +959,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Local 4*</t>
+          <t>%Local 2*</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ohms</t>
+          <t>Proportion</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>purple</t>
+          <t>blue</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>EIT Impedance</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>percentage</t>
         </is>
       </c>
     </row>
@@ -1016,7 +991,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>%Local 1*</t>
+          <t>%Local 3*</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1026,17 +1001,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>EIT Impedance</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>fraction</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1018,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>%Local 2*</t>
+          <t>%Local 4*</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1058,71 +1028,62 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>purple</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>EIT Impedance</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>percentage</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>eit</t>
+          <t>servo_u</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>%Local 3*</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Proportion</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>EIT Impedance</t>
-        </is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>eit</t>
+          <t>servo_u</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>%Local 4*</t>
+          <t>Airway Press. (cmH2O)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Airway Pressure</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Proportion</t>
+          <t>cmH2O</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>purple</t>
+          <t>#e74c3c</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>EIT Impedance</t>
+          <t>Pressure &amp; Flow</t>
         </is>
       </c>
     </row>
@@ -1134,14 +1095,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0.02</v>
+          <t>Volume (ml)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>mL</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>#3498db</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1152,22 +1127,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Airway Press. (cmH2O)</t>
+          <t>Airway Flow (ml / s)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Airway Pressure</t>
+          <t>Airway Flow</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>cmH2O</t>
-        </is>
+          <t>L/min</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.06</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>#e74c3c</t>
+          <t>#2ecc71</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1184,99 +1162,92 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Volume (ml)</t>
+          <t>Esophageal Press. (cmH2O)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Esophageal Pressure</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>mL</t>
+          <t>cmH2O</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>#3498db</t>
+          <t>#e74c3c</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>dash</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Volume</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>servo_u</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Airway Flow (ml / s)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Airway Flow</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>L/min</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>#2ecc71</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Pressure &amp; Flow</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>servo_u</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Esophageal Press. (cmH2O)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
           <t>Esophageal Pressure</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>cmH2O</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>#e74c3c</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>dash</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Esophageal Pressure</t>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mindray_scope</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>mindray_scope</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ECG_II</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ECG II</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>mV</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>#2c3e50</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Waveform</t>
         </is>
       </c>
     </row>
@@ -1288,14 +1259,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0.2</v>
+          <t>Pleth</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Plethysmography</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>#7d3c98</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Waveform</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1306,27 +1291,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ECG_II</t>
+          <t>Art</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ECG II</t>
+          <t>Arterial Pressure</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>mV</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>#2c3e50</t>
+          <t>mmHg</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Waveform</t>
+          <t>Arterial Pressure</t>
         </is>
       </c>
     </row>
@@ -1338,27 +1318,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pleth</t>
+          <t>Paw</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Plethysmography</t>
+          <t>Airway Pressure</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>cmH2O</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>#7d3c98</t>
+          <t>#e67e22</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Waveform</t>
+          <t>Pressure &amp; Flow</t>
         </is>
       </c>
     </row>
@@ -1370,22 +1350,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Art</t>
+          <t>Vol</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Arterial Pressure</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>mmHg</t>
+          <t>mL</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>#2471a3</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Arterial Pressure</t>
+          <t>Volume</t>
         </is>
       </c>
     </row>
@@ -1397,22 +1382,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Paw</t>
+          <t>debit</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Airway Pressure</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>cmH2O</t>
+          <t>L/min</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>#e67e22</t>
+          <t>#1e8449</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -1429,86 +1414,76 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vol</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Port 4 Pressure</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>mL</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>#2471a3</t>
+          <t>cmH2O</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Esophageal Pressure</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>mindray_scope</t>
+          <t>edf</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>debit</t>
+          <t>chan 1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>EEG 1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>L/min</t>
+          <t>µV</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>#1e8449</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Pressure &amp; Flow</t>
+          <t>steelblue</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>mindray_scope</t>
+          <t>edf</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>chan 2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Port 4 Pressure</t>
+          <t>EEG 2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>cmH2O</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>Esophageal Pressure</t>
+          <t>µV</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>darkorange</t>
         </is>
       </c>
     </row>
@@ -1520,12 +1495,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>chan 1</t>
+          <t>chan 3</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>EEG 1</t>
+          <t>EEG 3</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1534,60 +1509,6 @@
         </is>
       </c>
       <c r="I47" t="inlineStr">
-        <is>
-          <t>steelblue</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>edf</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>chan 2</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>EEG 2</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>µV</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>darkorange</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>edf</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>chan 3</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>EEG 3</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>µV</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
         <is>
           <t>seagreen</t>
         </is>

</xml_diff>

<commit_message>
Review for sdandar and maintainability
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="signals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loops" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spectrograms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="psds" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="signals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="loops" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="spectrograms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="psds" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1219,16 +1219,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -2612,7 +2602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2750,6 +2740,28 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>MDC_VOL_AWAY-MDC_DIM_MILLI_L</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PV loop cross-device (servo-u P, mindray V)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>servo_u::Airway Press. (cmH2O)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mindray_scope::Vol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed bug abotu spectral computation
</commit_message>
<xml_diff>
--- a/example/demo_database/database_options.xlsx
+++ b/example/demo_database/database_options.xlsx
@@ -2853,10 +2853,10 @@
         <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -2882,10 +2882,10 @@
         <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -2911,10 +2911,10 @@
         <v>30</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>

</xml_diff>